<commit_message>
Update on README and data files, new notebook and output tables
</commit_message>
<xml_diff>
--- a/data_raw/variable_metadata.xlsx
+++ b/data_raw/variable_metadata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://node9387-my.sharepoint.com/personal/toby_node9_co_uk/Documents/Documents/College &amp; Uni/Data Science Degree/Year Three/WBP/CSLS_Project/data_raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://node9387-my.sharepoint.com/personal/toby_node9_co_uk/Documents/Local Github Repo/CSBS Project/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FDB66D1-A86E-46C8-BC7B-41BA9DA48893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{7FDB66D1-A86E-46C8-BC7B-41BA9DA48893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D02DF20E-2772-4B9C-99DE-8AE594F0160B}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{98CA4F05-AB97-4F9C-9E8C-202B5E24FE7E}"/>
+    <workbookView xWindow="7929" yWindow="4637" windowWidth="24685" windowHeight="13054" xr2:uid="{98CA4F05-AB97-4F9C-9E8C-202B5E24FE7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Variable_Metadata" sheetId="1" r:id="rId1"/>
@@ -3354,34 +3354,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F143D036-95BC-4AF3-8B39-7C9E5165CF48}" name="Table10" displayName="Table10" ref="A1:H528" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:H528" xr:uid="{3F22AC71-F5F0-42C7-A3DA-AC10C980D9C3}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="questtype"/>
-        <filter val="samptype"/>
-        <filter val="type_comb1"/>
-        <filter val="type_comb2"/>
-        <filter val="type1"/>
-        <filter val="type10"/>
-        <filter val="type11"/>
-        <filter val="type12"/>
-        <filter val="type13"/>
-        <filter val="type15"/>
-        <filter val="type16"/>
-        <filter val="type2"/>
-        <filter val="type3"/>
-        <filter val="type4"/>
-        <filter val="type5"/>
-        <filter val="type6"/>
-        <filter val="type6x"/>
-        <filter val="type7"/>
-        <filter val="type8"/>
-        <filter val="type9"/>
-        <filter val="typex"/>
-        <filter val="typex_comb"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H528" xr:uid="{3F22AC71-F5F0-42C7-A3DA-AC10C980D9C3}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{75BB27AE-6661-48F8-AC7F-F1D32ACFCAC9}" name="Position"/>
     <tableColumn id="2" xr3:uid="{95A4CCC4-E4A2-4055-8A3D-128DC68DE65D}" name="VAR_ID"/>
@@ -3752,7 +3725,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3812,7 +3785,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>6</v>
       </c>
@@ -3835,7 +3808,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>10</v>
       </c>
@@ -3858,7 +3831,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>13</v>
       </c>
@@ -3881,7 +3854,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>15</v>
       </c>
@@ -3904,7 +3877,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>18</v>
       </c>
@@ -3927,7 +3900,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>26</v>
       </c>
@@ -3950,7 +3923,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>27</v>
       </c>
@@ -3973,7 +3946,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>28</v>
       </c>
@@ -3996,7 +3969,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>29</v>
       </c>
@@ -4019,7 +3992,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>30</v>
       </c>
@@ -4042,7 +4015,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>31</v>
       </c>
@@ -4065,7 +4038,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>32</v>
       </c>
@@ -4088,7 +4061,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>33</v>
       </c>
@@ -4111,7 +4084,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>34</v>
       </c>
@@ -4134,7 +4107,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>35</v>
       </c>
@@ -4157,7 +4130,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>36</v>
       </c>
@@ -4180,7 +4153,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>37</v>
       </c>
@@ -4203,7 +4176,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>38</v>
       </c>
@@ -4226,7 +4199,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>39</v>
       </c>
@@ -4249,7 +4222,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>40</v>
       </c>
@@ -4272,7 +4245,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>41</v>
       </c>
@@ -4295,7 +4268,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>42</v>
       </c>
@@ -4318,7 +4291,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>43</v>
       </c>
@@ -4341,7 +4314,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>44</v>
       </c>
@@ -4364,7 +4337,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>45</v>
       </c>
@@ -4387,7 +4360,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>46</v>
       </c>
@@ -4410,7 +4383,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>47</v>
       </c>
@@ -4433,7 +4406,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A32">
         <v>48</v>
       </c>
@@ -4456,7 +4429,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>49</v>
       </c>
@@ -4479,7 +4452,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>50</v>
       </c>
@@ -4502,7 +4475,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>51</v>
       </c>
@@ -4525,7 +4498,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>52</v>
       </c>
@@ -4548,7 +4521,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A37">
         <v>53</v>
       </c>
@@ -4571,7 +4544,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A38">
         <v>54</v>
       </c>
@@ -4594,7 +4567,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>55</v>
       </c>
@@ -4617,7 +4590,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>56</v>
       </c>
@@ -4640,7 +4613,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>57</v>
       </c>
@@ -4663,7 +4636,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>58</v>
       </c>
@@ -4686,7 +4659,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A43">
         <v>59</v>
       </c>
@@ -4709,7 +4682,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A44">
         <v>60</v>
       </c>
@@ -4732,7 +4705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A45">
         <v>61</v>
       </c>
@@ -4755,7 +4728,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A46">
         <v>62</v>
       </c>
@@ -4778,7 +4751,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A47">
         <v>63</v>
       </c>
@@ -4801,7 +4774,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>64</v>
       </c>
@@ -4824,7 +4797,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A49">
         <v>65</v>
       </c>
@@ -4847,7 +4820,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>66</v>
       </c>
@@ -4870,7 +4843,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>67</v>
       </c>
@@ -4893,7 +4866,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A52">
         <v>68</v>
       </c>
@@ -4916,7 +4889,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A53">
         <v>69</v>
       </c>
@@ -4939,7 +4912,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>168</v>
       </c>
@@ -4962,7 +4935,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A55">
         <v>169</v>
       </c>
@@ -4985,7 +4958,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>170</v>
       </c>
@@ -5008,7 +4981,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A57">
         <v>171</v>
       </c>
@@ -5031,7 +5004,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A58">
         <v>172</v>
       </c>
@@ -5054,7 +5027,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A59">
         <v>173</v>
       </c>
@@ -5077,7 +5050,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A60">
         <v>182</v>
       </c>
@@ -5100,7 +5073,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A61">
         <v>183</v>
       </c>
@@ -5123,7 +5096,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A62">
         <v>184</v>
       </c>
@@ -5146,7 +5119,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A63">
         <v>185</v>
       </c>
@@ -5169,7 +5142,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A64">
         <v>192</v>
       </c>
@@ -5192,7 +5165,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A65">
         <v>193</v>
       </c>
@@ -5215,7 +5188,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A66">
         <v>194</v>
       </c>
@@ -5238,7 +5211,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A67">
         <v>195</v>
       </c>
@@ -5261,7 +5234,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A68">
         <v>196</v>
       </c>
@@ -5284,7 +5257,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A69">
         <v>197</v>
       </c>
@@ -5307,7 +5280,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A70">
         <v>198</v>
       </c>
@@ -5330,7 +5303,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A71">
         <v>199</v>
       </c>
@@ -5353,7 +5326,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A72">
         <v>200</v>
       </c>
@@ -5376,7 +5349,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A73">
         <v>201</v>
       </c>
@@ -5399,7 +5372,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A74">
         <v>202</v>
       </c>
@@ -5422,7 +5395,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A75">
         <v>203</v>
       </c>
@@ -5445,7 +5418,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A76">
         <v>211</v>
       </c>
@@ -5468,7 +5441,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A77">
         <v>212</v>
       </c>
@@ -5491,7 +5464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A78">
         <v>213</v>
       </c>
@@ -5514,7 +5487,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A79">
         <v>214</v>
       </c>
@@ -5537,7 +5510,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A80">
         <v>215</v>
       </c>
@@ -5560,7 +5533,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A81">
         <v>216</v>
       </c>
@@ -5583,7 +5556,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A82">
         <v>217</v>
       </c>
@@ -5882,7 +5855,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A95">
         <v>259</v>
       </c>
@@ -5905,7 +5878,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A96">
         <v>261</v>
       </c>
@@ -5928,7 +5901,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A97">
         <v>262</v>
       </c>
@@ -5951,7 +5924,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A98">
         <v>263</v>
       </c>
@@ -5974,7 +5947,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A99">
         <v>264</v>
       </c>
@@ -5997,7 +5970,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A100">
         <v>265</v>
       </c>
@@ -6020,7 +5993,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A101">
         <v>266</v>
       </c>
@@ -6043,7 +6016,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A102">
         <v>267</v>
       </c>
@@ -6066,7 +6039,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A103">
         <v>268</v>
       </c>
@@ -6089,7 +6062,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A104">
         <v>269</v>
       </c>
@@ -6112,7 +6085,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A105">
         <v>270</v>
       </c>
@@ -6135,7 +6108,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A106">
         <v>275</v>
       </c>
@@ -6158,7 +6131,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A107">
         <v>276</v>
       </c>
@@ -6181,7 +6154,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A108">
         <v>277</v>
       </c>
@@ -6204,7 +6177,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A109">
         <v>278</v>
       </c>
@@ -6227,7 +6200,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A110">
         <v>279</v>
       </c>
@@ -6250,7 +6223,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A111">
         <v>280</v>
       </c>
@@ -6273,7 +6246,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A112">
         <v>281</v>
       </c>
@@ -6296,7 +6269,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A113">
         <v>282</v>
       </c>
@@ -6319,7 +6292,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A114">
         <v>283</v>
       </c>
@@ -6342,7 +6315,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A115">
         <v>284</v>
       </c>
@@ -6365,7 +6338,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A116">
         <v>285</v>
       </c>
@@ -6388,7 +6361,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A117">
         <v>286</v>
       </c>
@@ -6411,7 +6384,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A118">
         <v>287</v>
       </c>
@@ -6434,7 +6407,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A119">
         <v>309</v>
       </c>
@@ -6457,7 +6430,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A120">
         <v>311</v>
       </c>
@@ -6480,7 +6453,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A121">
         <v>325</v>
       </c>
@@ -6503,7 +6476,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A122">
         <v>326</v>
       </c>
@@ -6526,7 +6499,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A123">
         <v>327</v>
       </c>
@@ -6549,7 +6522,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A124">
         <v>328</v>
       </c>
@@ -6572,7 +6545,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A125">
         <v>329</v>
       </c>
@@ -6595,7 +6568,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A126">
         <v>330</v>
       </c>
@@ -6618,7 +6591,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A127">
         <v>331</v>
       </c>
@@ -6641,7 +6614,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A128">
         <v>332</v>
       </c>
@@ -6664,7 +6637,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A129">
         <v>333</v>
       </c>
@@ -6687,7 +6660,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A130">
         <v>334</v>
       </c>
@@ -6710,7 +6683,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A131">
         <v>335</v>
       </c>
@@ -6733,7 +6706,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A132">
         <v>336</v>
       </c>
@@ -6756,7 +6729,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A133">
         <v>337</v>
       </c>
@@ -6779,7 +6752,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A134">
         <v>338</v>
       </c>
@@ -6802,7 +6775,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A135">
         <v>339</v>
       </c>
@@ -6825,7 +6798,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A136">
         <v>340</v>
       </c>
@@ -6848,7 +6821,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A137">
         <v>341</v>
       </c>
@@ -6871,7 +6844,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A138">
         <v>342</v>
       </c>
@@ -6894,7 +6867,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A139">
         <v>343</v>
       </c>
@@ -6917,7 +6890,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A140">
         <v>344</v>
       </c>
@@ -6940,7 +6913,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A141">
         <v>350</v>
       </c>
@@ -6963,7 +6936,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A142">
         <v>351</v>
       </c>
@@ -6986,7 +6959,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A143">
         <v>352</v>
       </c>
@@ -7009,7 +6982,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A144">
         <v>353</v>
       </c>
@@ -7032,7 +7005,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A145">
         <v>354</v>
       </c>
@@ -7055,7 +7028,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="146" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A146">
         <v>355</v>
       </c>
@@ -7078,7 +7051,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="147" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A147">
         <v>356</v>
       </c>
@@ -7101,7 +7074,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="148" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A148">
         <v>357</v>
       </c>
@@ -7124,7 +7097,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="149" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A149">
         <v>358</v>
       </c>
@@ -7147,7 +7120,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A150">
         <v>359</v>
       </c>
@@ -7170,7 +7143,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="151" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A151">
         <v>360</v>
       </c>
@@ -7193,7 +7166,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="152" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A152">
         <v>361</v>
       </c>
@@ -7216,7 +7189,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A153">
         <v>362</v>
       </c>
@@ -7239,7 +7212,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A154">
         <v>363</v>
       </c>
@@ -7262,7 +7235,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="155" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="155" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A155">
         <v>364</v>
       </c>
@@ -7285,7 +7258,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="156" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="156" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A156">
         <v>365</v>
       </c>
@@ -7308,7 +7281,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="157" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="157" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A157">
         <v>366</v>
       </c>
@@ -7331,7 +7304,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="158" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="158" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A158">
         <v>367</v>
       </c>
@@ -7354,7 +7327,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="159" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="159" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A159">
         <v>368</v>
       </c>
@@ -7377,7 +7350,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="160" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A160">
         <v>491</v>
       </c>
@@ -7403,7 +7376,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A161">
         <v>492</v>
       </c>
@@ -7429,7 +7402,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="162" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="162" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A162">
         <v>493</v>
       </c>
@@ -7455,7 +7428,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="163" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="163" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A163">
         <v>494</v>
       </c>
@@ -7481,7 +7454,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="164" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A164">
         <v>495</v>
       </c>
@@ -7507,7 +7480,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A165">
         <v>496</v>
       </c>
@@ -7533,7 +7506,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="166" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A166">
         <v>497</v>
       </c>
@@ -7559,7 +7532,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="167" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A167">
         <v>498</v>
       </c>
@@ -7585,7 +7558,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="168" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A168">
         <v>499</v>
       </c>
@@ -7611,7 +7584,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="169" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A169">
         <v>500</v>
       </c>
@@ -7637,7 +7610,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="170" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="170" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A170">
         <v>501</v>
       </c>
@@ -7663,7 +7636,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A171">
         <v>502</v>
       </c>
@@ -7689,7 +7662,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A172">
         <v>503</v>
       </c>
@@ -7715,7 +7688,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A173">
         <v>504</v>
       </c>
@@ -7741,7 +7714,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A174">
         <v>527</v>
       </c>
@@ -7784,7 +7757,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A176">
         <v>5</v>
       </c>
@@ -7807,7 +7780,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="177" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A177">
         <v>204</v>
       </c>
@@ -7830,7 +7803,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="178" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A178">
         <v>223</v>
       </c>
@@ -7853,7 +7826,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A179">
         <v>345</v>
       </c>
@@ -7876,7 +7849,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="180" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A180">
         <v>70</v>
       </c>
@@ -7899,7 +7872,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A181">
         <v>109</v>
       </c>
@@ -7922,7 +7895,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="182" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A182">
         <v>110</v>
       </c>
@@ -7945,7 +7918,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="183" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A183">
         <v>111</v>
       </c>
@@ -7968,7 +7941,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="184" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A184">
         <v>112</v>
       </c>
@@ -7991,7 +7964,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A185">
         <v>113</v>
       </c>
@@ -8014,7 +7987,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="186" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="186" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A186">
         <v>186</v>
       </c>
@@ -8037,7 +8010,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="187" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="187" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A187">
         <v>205</v>
       </c>
@@ -8060,7 +8033,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="188" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="188" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A188">
         <v>231</v>
       </c>
@@ -8083,7 +8056,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="189" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A189">
         <v>232</v>
       </c>
@@ -8129,7 +8102,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="191" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="191" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A191">
         <v>385</v>
       </c>
@@ -8152,7 +8125,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="192" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="192" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A192">
         <v>386</v>
       </c>
@@ -8175,7 +8148,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="193" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="193" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A193">
         <v>387</v>
       </c>
@@ -8198,7 +8171,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="194" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="194" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A194">
         <v>388</v>
       </c>
@@ -8221,7 +8194,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="195" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="195" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A195">
         <v>389</v>
       </c>
@@ -8244,7 +8217,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="196" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="196" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A196">
         <v>71</v>
       </c>
@@ -8267,7 +8240,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="197" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="197" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A197">
         <v>72</v>
       </c>
@@ -8290,7 +8263,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="198" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="198" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A198">
         <v>73</v>
       </c>
@@ -8313,7 +8286,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="199" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="199" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A199">
         <v>74</v>
       </c>
@@ -8336,7 +8309,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="200" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="200" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A200">
         <v>75</v>
       </c>
@@ -8359,7 +8332,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="201" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="201" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A201">
         <v>76</v>
       </c>
@@ -8382,7 +8355,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="202" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="202" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A202">
         <v>77</v>
       </c>
@@ -8405,7 +8378,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="203" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="203" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A203">
         <v>78</v>
       </c>
@@ -8428,7 +8401,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="204" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="204" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A204">
         <v>79</v>
       </c>
@@ -8451,7 +8424,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="205" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="205" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A205">
         <v>80</v>
       </c>
@@ -8474,7 +8447,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="206" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="206" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A206">
         <v>81</v>
       </c>
@@ -8497,7 +8470,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="207" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="207" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A207">
         <v>82</v>
       </c>
@@ -8520,7 +8493,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="208" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="208" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A208">
         <v>83</v>
       </c>
@@ -8543,7 +8516,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="209" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="209" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A209">
         <v>118</v>
       </c>
@@ -8566,7 +8539,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="210" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="210" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A210">
         <v>119</v>
       </c>
@@ -8589,7 +8562,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="211" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="211" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A211">
         <v>120</v>
       </c>
@@ -8612,7 +8585,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="212" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="212" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A212">
         <v>121</v>
       </c>
@@ -8635,7 +8608,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="213" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="213" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A213">
         <v>122</v>
       </c>
@@ -8658,7 +8631,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="214" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="214" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A214">
         <v>123</v>
       </c>
@@ -8681,7 +8654,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="215" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="215" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A215">
         <v>124</v>
       </c>
@@ -8704,7 +8677,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="216" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="216" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A216">
         <v>125</v>
       </c>
@@ -8727,7 +8700,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="217" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="217" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A217">
         <v>126</v>
       </c>
@@ -8750,7 +8723,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="218" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="218" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A218">
         <v>127</v>
       </c>
@@ -8773,7 +8746,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="219" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="219" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A219">
         <v>128</v>
       </c>
@@ -8796,7 +8769,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="220" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="220" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A220">
         <v>129</v>
       </c>
@@ -8819,7 +8792,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="221" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="221" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A221">
         <v>130</v>
       </c>
@@ -8842,7 +8815,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="222" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="222" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A222">
         <v>131</v>
       </c>
@@ -8865,7 +8838,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="223" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="223" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A223">
         <v>132</v>
       </c>
@@ -8888,7 +8861,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="224" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="224" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A224">
         <v>133</v>
       </c>
@@ -8911,7 +8884,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="225" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="225" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A225">
         <v>134</v>
       </c>
@@ -8934,7 +8907,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="226" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="226" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A226">
         <v>135</v>
       </c>
@@ -8957,7 +8930,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="227" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="227" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A227">
         <v>136</v>
       </c>
@@ -8980,7 +8953,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="228" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="228" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A228">
         <v>137</v>
       </c>
@@ -9003,7 +8976,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="229" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="229" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A229">
         <v>138</v>
       </c>
@@ -9026,7 +8999,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="230" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="230" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A230">
         <v>139</v>
       </c>
@@ -9049,7 +9022,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="231" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="231" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A231">
         <v>140</v>
       </c>
@@ -9072,7 +9045,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="232" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="232" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A232">
         <v>141</v>
       </c>
@@ -9095,7 +9068,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="233" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="233" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A233">
         <v>142</v>
       </c>
@@ -9118,7 +9091,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="234" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="234" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A234">
         <v>143</v>
       </c>
@@ -9141,7 +9114,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="235" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="235" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A235">
         <v>144</v>
       </c>
@@ -9164,7 +9137,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="236" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="236" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A236">
         <v>145</v>
       </c>
@@ -9187,7 +9160,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="237" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="237" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A237">
         <v>146</v>
       </c>
@@ -9210,7 +9183,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="238" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="238" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A238">
         <v>147</v>
       </c>
@@ -9233,7 +9206,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="239" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="239" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A239">
         <v>148</v>
       </c>
@@ -9256,7 +9229,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="240" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="240" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A240">
         <v>149</v>
       </c>
@@ -9279,7 +9252,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="241" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="241" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A241">
         <v>150</v>
       </c>
@@ -9302,7 +9275,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="242" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="242" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A242">
         <v>151</v>
       </c>
@@ -9325,7 +9298,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="243" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="243" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A243">
         <v>152</v>
       </c>
@@ -9348,7 +9321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="244" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="244" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A244">
         <v>153</v>
       </c>
@@ -9371,7 +9344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="245" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="245" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A245">
         <v>154</v>
       </c>
@@ -9394,7 +9367,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="246" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="246" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A246">
         <v>155</v>
       </c>
@@ -9417,7 +9390,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="247" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="247" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A247">
         <v>156</v>
       </c>
@@ -9440,7 +9413,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="248" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="248" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A248">
         <v>157</v>
       </c>
@@ -9463,7 +9436,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="249" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="249" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A249">
         <v>158</v>
       </c>
@@ -9486,7 +9459,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="250" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="250" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A250">
         <v>159</v>
       </c>
@@ -9509,7 +9482,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="251" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="251" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A251">
         <v>176</v>
       </c>
@@ -9532,7 +9505,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="252" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="252" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A252">
         <v>177</v>
       </c>
@@ -9555,7 +9528,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="253" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="253" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A253">
         <v>178</v>
       </c>
@@ -9578,7 +9551,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="254" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="254" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A254">
         <v>179</v>
       </c>
@@ -9601,7 +9574,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="255" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="255" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A255">
         <v>180</v>
       </c>
@@ -9624,7 +9597,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="256" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="256" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A256">
         <v>187</v>
       </c>
@@ -9647,7 +9620,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="257" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="257" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A257">
         <v>188</v>
       </c>
@@ -9670,7 +9643,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="258" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="258" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A258">
         <v>189</v>
       </c>
@@ -9693,7 +9666,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="259" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A259">
         <v>191</v>
       </c>
@@ -9716,7 +9689,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="260" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="260" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A260">
         <v>206</v>
       </c>
@@ -9739,7 +9712,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="261" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="261" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A261">
         <v>207</v>
       </c>
@@ -9762,7 +9735,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="262" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="262" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A262">
         <v>218</v>
       </c>
@@ -9785,7 +9758,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="263" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="263" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A263">
         <v>219</v>
       </c>
@@ -9808,7 +9781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="264" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="264" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A264">
         <v>226</v>
       </c>
@@ -9877,7 +9850,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="267" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="267" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A267">
         <v>271</v>
       </c>
@@ -9900,7 +9873,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="268" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="268" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A268">
         <v>272</v>
       </c>
@@ -9923,7 +9896,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="269" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="269" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A269">
         <v>273</v>
       </c>
@@ -9946,7 +9919,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="270" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="270" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A270">
         <v>369</v>
       </c>
@@ -9969,7 +9942,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="271" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="271" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A271">
         <v>370</v>
       </c>
@@ -9992,7 +9965,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="272" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="272" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A272">
         <v>371</v>
       </c>
@@ -10015,7 +9988,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="273" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="273" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A273">
         <v>372</v>
       </c>
@@ -10038,7 +10011,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="274" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="274" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A274">
         <v>373</v>
       </c>
@@ -10061,7 +10034,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="275" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="275" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A275">
         <v>374</v>
       </c>
@@ -10084,7 +10057,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="276" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="276" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A276">
         <v>375</v>
       </c>
@@ -10107,7 +10080,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="277" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="277" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A277">
         <v>376</v>
       </c>
@@ -10130,7 +10103,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="278" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="278" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A278">
         <v>377</v>
       </c>
@@ -10153,7 +10126,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="279" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="279" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A279">
         <v>378</v>
       </c>
@@ -10176,7 +10149,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="280" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="280" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A280">
         <v>487</v>
       </c>
@@ -10202,7 +10175,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="281" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="281" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A281">
         <v>488</v>
       </c>
@@ -10228,7 +10201,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="282" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A282">
         <v>489</v>
       </c>
@@ -10254,7 +10227,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="283" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A283">
         <v>490</v>
       </c>
@@ -10280,7 +10253,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="284" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A284">
         <v>7</v>
       </c>
@@ -10303,7 +10276,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="285" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="285" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A285">
         <v>98</v>
       </c>
@@ -10326,7 +10299,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="286" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="286" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A286">
         <v>99</v>
       </c>
@@ -10349,7 +10322,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="287" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="287" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A287">
         <v>84</v>
       </c>
@@ -10372,7 +10345,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="288" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="288" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A288">
         <v>174</v>
       </c>
@@ -10395,7 +10368,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="289" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="289" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A289">
         <v>208</v>
       </c>
@@ -10418,7 +10391,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="290" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="290" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A290">
         <v>227</v>
       </c>
@@ -10441,7 +10414,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="291" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="291" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A291">
         <v>228</v>
       </c>
@@ -10464,7 +10437,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="292" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A292">
         <v>229</v>
       </c>
@@ -10487,7 +10460,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="293" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A293">
         <v>230</v>
       </c>
@@ -10510,7 +10483,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="294" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A294">
         <v>346</v>
       </c>
@@ -10533,7 +10506,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="295" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="295" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A295">
         <v>390</v>
       </c>
@@ -10556,7 +10529,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="296" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="296" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A296">
         <v>391</v>
       </c>
@@ -10579,7 +10552,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="297" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="297" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A297">
         <v>392</v>
       </c>
@@ -10602,7 +10575,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="298" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="298" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A298">
         <v>393</v>
       </c>
@@ -10625,7 +10598,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="299" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="299" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A299">
         <v>394</v>
       </c>
@@ -10648,7 +10621,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="300" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="300" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A300">
         <v>395</v>
       </c>
@@ -10671,7 +10644,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="301" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="301" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A301">
         <v>396</v>
       </c>
@@ -10694,7 +10667,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="302" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="302" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A302">
         <v>397</v>
       </c>
@@ -10717,7 +10690,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="303" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="303" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A303">
         <v>398</v>
       </c>
@@ -10740,7 +10713,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="304" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="304" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A304">
         <v>222</v>
       </c>
@@ -10763,7 +10736,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="305" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A305">
         <v>4</v>
       </c>
@@ -10786,7 +10759,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="306" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="306" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A306">
         <v>85</v>
       </c>
@@ -10809,7 +10782,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="307" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="307" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A307">
         <v>86</v>
       </c>
@@ -10832,7 +10805,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="308" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="308" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A308">
         <v>87</v>
       </c>
@@ -10855,7 +10828,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="309" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="309" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A309">
         <v>88</v>
       </c>
@@ -10878,7 +10851,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="310" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="310" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A310">
         <v>89</v>
       </c>
@@ -10901,7 +10874,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="311" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="311" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A311">
         <v>90</v>
       </c>
@@ -10924,7 +10897,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="312" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="312" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A312">
         <v>91</v>
       </c>
@@ -10947,7 +10920,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="313" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="313" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A313">
         <v>92</v>
       </c>
@@ -10970,7 +10943,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="314" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="314" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A314">
         <v>93</v>
       </c>
@@ -10993,7 +10966,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="315" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="315" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A315">
         <v>94</v>
       </c>
@@ -11016,7 +10989,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="316" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="316" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A316">
         <v>95</v>
       </c>
@@ -11039,7 +11012,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="317" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="317" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A317">
         <v>96</v>
       </c>
@@ -11062,7 +11035,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="318" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="318" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A318">
         <v>97</v>
       </c>
@@ -11085,7 +11058,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="319" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="319" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A319">
         <v>114</v>
       </c>
@@ -11108,7 +11081,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="320" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="320" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A320">
         <v>160</v>
       </c>
@@ -11131,7 +11104,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="321" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="321" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A321">
         <v>161</v>
       </c>
@@ -11154,7 +11127,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="322" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="322" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A322">
         <v>162</v>
       </c>
@@ -11177,7 +11150,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="323" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="323" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A323">
         <v>163</v>
       </c>
@@ -11200,7 +11173,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="324" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="324" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A324">
         <v>312</v>
       </c>
@@ -11223,7 +11196,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="325" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="325" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A325">
         <v>313</v>
       </c>
@@ -11246,7 +11219,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="326" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="326" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A326">
         <v>314</v>
       </c>
@@ -11269,7 +11242,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="327" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="327" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A327">
         <v>315</v>
       </c>
@@ -11292,7 +11265,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="328" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="328" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A328">
         <v>316</v>
       </c>
@@ -11315,7 +11288,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="329" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="329" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A329">
         <v>317</v>
       </c>
@@ -11338,7 +11311,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="330" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="330" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A330">
         <v>318</v>
       </c>
@@ -11361,7 +11334,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="331" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="331" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A331">
         <v>319</v>
       </c>
@@ -11384,7 +11357,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="332" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="332" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A332">
         <v>320</v>
       </c>
@@ -11407,7 +11380,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="333" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="333" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A333">
         <v>321</v>
       </c>
@@ -11430,7 +11403,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="334" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="334" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A334">
         <v>322</v>
       </c>
@@ -11453,7 +11426,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="335" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="335" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A335">
         <v>323</v>
       </c>
@@ -11476,7 +11449,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="336" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="336" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A336">
         <v>324</v>
       </c>
@@ -11499,7 +11472,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="337" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="337" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A337">
         <v>379</v>
       </c>
@@ -11522,7 +11495,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="338" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="338" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A338">
         <v>432</v>
       </c>
@@ -11545,7 +11518,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="339" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="339" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A339">
         <v>436</v>
       </c>
@@ -11568,7 +11541,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="340" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="340" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A340">
         <v>475</v>
       </c>
@@ -11591,7 +11564,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="341" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="341" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A341">
         <v>439</v>
       </c>
@@ -11614,7 +11587,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="342" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="342" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A342">
         <v>443</v>
       </c>
@@ -11637,7 +11610,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="343" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="343" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A343">
         <v>446</v>
       </c>
@@ -11660,7 +11633,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="344" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="344" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A344">
         <v>450</v>
       </c>
@@ -11683,7 +11656,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="345" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="345" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A345">
         <v>454</v>
       </c>
@@ -11706,7 +11679,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="346" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="346" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A346">
         <v>457</v>
       </c>
@@ -11729,7 +11702,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="347" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="347" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A347">
         <v>461</v>
       </c>
@@ -11752,7 +11725,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="348" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="348" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A348">
         <v>465</v>
       </c>
@@ -11775,7 +11748,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="349" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="349" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A349">
         <v>468</v>
       </c>
@@ -11798,7 +11771,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="350" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="350" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A350">
         <v>471</v>
       </c>
@@ -11821,7 +11794,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="351" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="351" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A351">
         <v>479</v>
       </c>
@@ -11844,7 +11817,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="352" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="352" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A352">
         <v>483</v>
       </c>
@@ -11867,7 +11840,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="353" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="353" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A353">
         <v>505</v>
       </c>
@@ -11893,7 +11866,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="354" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="354" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A354">
         <v>506</v>
       </c>
@@ -11919,7 +11892,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="355" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="355" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A355">
         <v>507</v>
       </c>
@@ -11945,7 +11918,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="356" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="356" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A356">
         <v>508</v>
       </c>
@@ -11971,7 +11944,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="357" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="357" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A357">
         <v>509</v>
       </c>
@@ -11997,7 +11970,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="358" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="358" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A358">
         <v>510</v>
       </c>
@@ -12023,7 +11996,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="359" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="359" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A359">
         <v>511</v>
       </c>
@@ -12049,7 +12022,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="360" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="360" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A360">
         <v>512</v>
       </c>
@@ -12075,7 +12048,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="361" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="361" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A361">
         <v>513</v>
       </c>
@@ -12101,7 +12074,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="362" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="362" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A362">
         <v>514</v>
       </c>
@@ -12127,7 +12100,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="363" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="363" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A363">
         <v>515</v>
       </c>
@@ -12153,7 +12126,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="364" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="364" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A364">
         <v>516</v>
       </c>
@@ -12179,7 +12152,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="365" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="365" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A365">
         <v>517</v>
       </c>
@@ -12205,7 +12178,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="366" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="366" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A366">
         <v>518</v>
       </c>
@@ -12231,7 +12204,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="367" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="367" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A367">
         <v>519</v>
       </c>
@@ -12257,7 +12230,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="368" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="368" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A368">
         <v>520</v>
       </c>
@@ -12283,7 +12256,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="369" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="369" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A369">
         <v>521</v>
       </c>
@@ -12309,7 +12282,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="370" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="370" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A370">
         <v>522</v>
       </c>
@@ -12335,7 +12308,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="371" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="371" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A371">
         <v>523</v>
       </c>
@@ -12361,7 +12334,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="372" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="372" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A372">
         <v>524</v>
       </c>
@@ -12387,7 +12360,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="373" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="373" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A373">
         <v>526</v>
       </c>
@@ -12413,7 +12386,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="374" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="374" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A374">
         <v>525</v>
       </c>
@@ -12462,7 +12435,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="376" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="376" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A376">
         <v>11</v>
       </c>
@@ -12485,7 +12458,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="377" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="377" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A377">
         <v>12</v>
       </c>
@@ -12508,7 +12481,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="378" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="378" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A378">
         <v>14</v>
       </c>
@@ -12531,7 +12504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="379" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="379" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A379">
         <v>16</v>
       </c>
@@ -12554,7 +12527,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="380" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="380" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A380">
         <v>17</v>
       </c>
@@ -12577,7 +12550,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="381" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="381" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A381">
         <v>19</v>
       </c>
@@ -12600,7 +12573,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="382" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="382" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A382">
         <v>100</v>
       </c>
@@ -12623,7 +12596,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="383" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="383" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A383">
         <v>101</v>
       </c>
@@ -12646,7 +12619,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="384" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="384" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A384">
         <v>102</v>
       </c>
@@ -12669,7 +12642,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="385" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="385" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A385">
         <v>103</v>
       </c>
@@ -12692,7 +12665,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="386" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="386" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A386">
         <v>104</v>
       </c>
@@ -12715,7 +12688,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="387" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="387" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A387">
         <v>105</v>
       </c>
@@ -12738,7 +12711,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="388" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="388" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A388">
         <v>106</v>
       </c>
@@ -12761,7 +12734,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="389" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="389" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A389">
         <v>107</v>
       </c>
@@ -12784,7 +12757,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="390" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="390" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A390">
         <v>108</v>
       </c>
@@ -12807,7 +12780,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="391" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="391" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A391">
         <v>115</v>
       </c>
@@ -12830,7 +12803,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="392" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="392" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A392">
         <v>116</v>
       </c>
@@ -12853,7 +12826,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="393" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="393" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A393">
         <v>117</v>
       </c>
@@ -12879,7 +12852,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="394" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="394" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A394">
         <v>164</v>
       </c>
@@ -12902,7 +12875,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="395" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="395" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A395">
         <v>165</v>
       </c>
@@ -12925,7 +12898,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="396" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="396" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A396">
         <v>166</v>
       </c>
@@ -12948,7 +12921,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="397" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="397" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A397">
         <v>167</v>
       </c>
@@ -12971,7 +12944,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="398" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="398" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A398">
         <v>175</v>
       </c>
@@ -12994,7 +12967,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="399" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="399" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A399">
         <v>190</v>
       </c>
@@ -13017,7 +12990,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="400" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="400" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A400">
         <v>209</v>
       </c>
@@ -13040,7 +13013,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="401" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="401" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A401">
         <v>210</v>
       </c>
@@ -13063,7 +13036,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="402" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="402" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A402">
         <v>220</v>
       </c>
@@ -13086,7 +13059,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="403" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="403" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A403">
         <v>221</v>
       </c>
@@ -13109,7 +13082,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="404" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="404" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A404">
         <v>224</v>
       </c>
@@ -13132,7 +13105,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="405" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="405" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A405">
         <v>225</v>
       </c>
@@ -13155,7 +13128,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="406" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="406" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A406">
         <v>233</v>
       </c>
@@ -13181,7 +13154,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="407" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="407" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A407">
         <v>234</v>
       </c>
@@ -13204,7 +13177,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="408" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="408" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A408">
         <v>235</v>
       </c>
@@ -13227,7 +13200,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="409" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="409" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A409">
         <v>236</v>
       </c>
@@ -13250,7 +13223,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="410" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="410" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A410">
         <v>237</v>
       </c>
@@ -13348,7 +13321,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="414" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="414" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A414">
         <v>256</v>
       </c>
@@ -13374,7 +13347,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="415" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="415" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A415">
         <v>257</v>
       </c>
@@ -13397,7 +13370,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="416" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="416" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A416">
         <v>258</v>
       </c>
@@ -13420,7 +13393,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="417" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="417" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A417">
         <v>260</v>
       </c>
@@ -13443,7 +13416,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="418" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="418" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A418">
         <v>289</v>
       </c>
@@ -13466,7 +13439,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="419" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="419" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A419">
         <v>290</v>
       </c>
@@ -13492,7 +13465,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="420" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="420" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A420">
         <v>310</v>
       </c>
@@ -13515,7 +13488,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="421" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="421" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A421">
         <v>347</v>
       </c>
@@ -13538,7 +13511,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="422" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="422" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A422">
         <v>348</v>
       </c>
@@ -13561,7 +13534,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="423" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="423" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A423">
         <v>349</v>
       </c>
@@ -13587,7 +13560,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="424" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="424" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A424">
         <v>381</v>
       </c>
@@ -13610,7 +13583,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="425" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="425" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A425">
         <v>382</v>
       </c>
@@ -13633,7 +13606,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="426" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="426" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A426">
         <v>383</v>
       </c>
@@ -13656,7 +13629,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="427" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="427" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A427">
         <v>384</v>
       </c>
@@ -13679,7 +13652,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="428" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="428" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A428">
         <v>399</v>
       </c>
@@ -13702,7 +13675,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="429" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="429" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A429">
         <v>400</v>
       </c>
@@ -13725,7 +13698,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="430" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="430" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A430">
         <v>401</v>
       </c>
@@ -13748,7 +13721,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="431" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="431" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A431">
         <v>402</v>
       </c>
@@ -13771,7 +13744,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="432" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="432" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A432">
         <v>403</v>
       </c>
@@ -13794,7 +13767,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="433" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="433" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A433">
         <v>404</v>
       </c>
@@ -13817,7 +13790,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="434" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="434" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A434">
         <v>405</v>
       </c>
@@ -13840,7 +13813,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="435" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="435" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A435">
         <v>406</v>
       </c>
@@ -13863,7 +13836,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="436" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="436" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A436">
         <v>407</v>
       </c>
@@ -13886,7 +13859,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="437" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="437" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A437">
         <v>408</v>
       </c>
@@ -13909,7 +13882,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="438" spans="1:7" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="438" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A438">
         <v>409</v>
       </c>
@@ -13932,7 +13905,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="439" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="439" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A439">
         <v>410</v>
       </c>
@@ -13955,7 +13928,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="440" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="440" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A440">
         <v>411</v>
       </c>
@@ -13978,7 +13951,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="441" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="441" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A441">
         <v>412</v>
       </c>
@@ -14001,7 +13974,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="442" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="442" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A442">
         <v>413</v>
       </c>
@@ -14024,7 +13997,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="443" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="443" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A443">
         <v>414</v>
       </c>
@@ -14047,7 +14020,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="444" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="444" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A444">
         <v>415</v>
       </c>
@@ -14070,7 +14043,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="445" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="445" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A445">
         <v>416</v>
       </c>
@@ -14093,7 +14066,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="446" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="446" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A446">
         <v>417</v>
       </c>
@@ -14116,7 +14089,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="447" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="447" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A447">
         <v>418</v>
       </c>
@@ -14139,7 +14112,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="448" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="448" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A448">
         <v>419</v>
       </c>
@@ -14162,7 +14135,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="449" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="449" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A449">
         <v>420</v>
       </c>
@@ -14185,7 +14158,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="450" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="450" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A450">
         <v>421</v>
       </c>
@@ -14208,7 +14181,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="451" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="451" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A451">
         <v>422</v>
       </c>
@@ -14231,7 +14204,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="452" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="452" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A452">
         <v>423</v>
       </c>
@@ -14254,7 +14227,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="453" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="453" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A453">
         <v>424</v>
       </c>
@@ -14277,7 +14250,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="454" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="454" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A454">
         <v>425</v>
       </c>
@@ -14300,7 +14273,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="455" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="455" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A455">
         <v>426</v>
       </c>
@@ -14323,7 +14296,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="456" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="456" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A456">
         <v>427</v>
       </c>
@@ -14346,7 +14319,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="457" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="457" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A457">
         <v>428</v>
       </c>
@@ -14369,7 +14342,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="458" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="458" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A458">
         <v>429</v>
       </c>
@@ -14392,7 +14365,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="459" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="459" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A459">
         <v>430</v>
       </c>
@@ -14418,7 +14391,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="460" spans="1:8" ht="43.75" hidden="1" x14ac:dyDescent="0.4">
+    <row r="460" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A460">
         <v>431</v>
       </c>
@@ -14441,7 +14414,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="461" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="461" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A461">
         <v>433</v>
       </c>
@@ -14467,7 +14440,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="462" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="462" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A462">
         <v>434</v>
       </c>
@@ -14490,7 +14463,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="463" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="463" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A463">
         <v>435</v>
       </c>
@@ -14516,7 +14489,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="464" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="464" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A464">
         <v>437</v>
       </c>
@@ -14542,7 +14515,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="465" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="465" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A465">
         <v>438</v>
       </c>
@@ -14568,7 +14541,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="466" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="466" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A466">
         <v>440</v>
       </c>
@@ -14591,7 +14564,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="467" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="467" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A467">
         <v>441</v>
       </c>
@@ -14617,7 +14590,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="468" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="468" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A468">
         <v>442</v>
       </c>
@@ -14640,7 +14613,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="469" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="469" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A469">
         <v>444</v>
       </c>
@@ -14666,7 +14639,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="470" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="470" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A470">
         <v>445</v>
       </c>
@@ -14689,7 +14662,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="471" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="471" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A471">
         <v>447</v>
       </c>
@@ -14715,7 +14688,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="472" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="472" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A472">
         <v>448</v>
       </c>
@@ -14738,7 +14711,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="473" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="473" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A473">
         <v>449</v>
       </c>
@@ -14764,7 +14737,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="474" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="474" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A474">
         <v>451</v>
       </c>
@@ -14787,7 +14760,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="475" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="475" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A475">
         <v>452</v>
       </c>
@@ -14813,7 +14786,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="476" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="476" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A476">
         <v>453</v>
       </c>
@@ -14836,7 +14809,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="477" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="477" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A477">
         <v>455</v>
       </c>
@@ -14862,7 +14835,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="478" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="478" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A478">
         <v>456</v>
       </c>
@@ -14885,7 +14858,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="479" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="479" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A479">
         <v>458</v>
       </c>
@@ -14911,7 +14884,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="480" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="480" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A480">
         <v>459</v>
       </c>
@@ -14934,7 +14907,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="481" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="481" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A481">
         <v>460</v>
       </c>
@@ -14960,7 +14933,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="482" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="482" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A482">
         <v>462</v>
       </c>
@@ -14983,7 +14956,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="483" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="483" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A483">
         <v>463</v>
       </c>
@@ -15009,7 +14982,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="484" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="484" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A484">
         <v>464</v>
       </c>
@@ -15032,7 +15005,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="485" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="485" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A485">
         <v>466</v>
       </c>
@@ -15058,7 +15031,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="486" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="486" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A486">
         <v>467</v>
       </c>
@@ -15081,7 +15054,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="487" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="487" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A487">
         <v>469</v>
       </c>
@@ -15107,7 +15080,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="488" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="488" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A488">
         <v>470</v>
       </c>
@@ -15130,7 +15103,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="489" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="489" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A489">
         <v>472</v>
       </c>
@@ -15156,7 +15129,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="490" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="490" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A490">
         <v>473</v>
       </c>
@@ -15179,7 +15152,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="491" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="491" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A491">
         <v>474</v>
       </c>
@@ -15205,7 +15178,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="492" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="492" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A492">
         <v>476</v>
       </c>
@@ -15231,7 +15204,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="493" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="493" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A493">
         <v>477</v>
       </c>
@@ -15254,7 +15227,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="494" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="494" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A494">
         <v>478</v>
       </c>
@@ -15280,7 +15253,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="495" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="495" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A495">
         <v>480</v>
       </c>
@@ -15306,7 +15279,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="496" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="496" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A496">
         <v>481</v>
       </c>
@@ -15329,7 +15302,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="497" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="497" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A497">
         <v>482</v>
       </c>
@@ -15352,7 +15325,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="498" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="498" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A498">
         <v>484</v>
       </c>
@@ -15375,7 +15348,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="499" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="499" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A499">
         <v>485</v>
       </c>
@@ -15401,7 +15374,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="500" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="500" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A500">
         <v>486</v>
       </c>
@@ -15424,7 +15397,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="501" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="501" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A501">
         <v>20</v>
       </c>
@@ -15447,7 +15420,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="502" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="502" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A502">
         <v>21</v>
       </c>
@@ -15470,7 +15443,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="503" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="503" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A503">
         <v>22</v>
       </c>
@@ -15493,7 +15466,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="504" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="504" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A504">
         <v>23</v>
       </c>
@@ -15516,7 +15489,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="505" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="505" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A505">
         <v>24</v>
       </c>
@@ -15539,7 +15512,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="506" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="506" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A506">
         <v>25</v>
       </c>
@@ -15562,7 +15535,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="507" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="507" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A507">
         <v>181</v>
       </c>
@@ -15585,7 +15558,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="508" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="508" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A508">
         <v>274</v>
       </c>
@@ -15611,7 +15584,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="509" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="509" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A509">
         <v>288</v>
       </c>
@@ -15634,7 +15607,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="510" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="510" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A510">
         <v>291</v>
       </c>
@@ -15657,7 +15630,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="511" spans="1:8" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="511" spans="1:8" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A511">
         <v>292</v>
       </c>
@@ -15680,7 +15653,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="512" spans="1:8" hidden="1" x14ac:dyDescent="0.4">
+    <row r="512" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A512">
         <v>293</v>
       </c>
@@ -15703,7 +15676,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="513" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="513" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A513">
         <v>294</v>
       </c>
@@ -15726,7 +15699,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="514" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="514" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A514">
         <v>295</v>
       </c>
@@ -15749,7 +15722,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="515" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="515" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A515">
         <v>296</v>
       </c>
@@ -15772,7 +15745,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="516" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="516" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A516">
         <v>297</v>
       </c>
@@ -15795,7 +15768,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="517" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="517" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A517">
         <v>298</v>
       </c>
@@ -15818,7 +15791,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="518" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="518" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A518">
         <v>299</v>
       </c>
@@ -15841,7 +15814,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="519" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="519" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A519">
         <v>300</v>
       </c>
@@ -15864,7 +15837,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="520" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="520" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A520">
         <v>301</v>
       </c>
@@ -15887,7 +15860,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="521" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="521" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A521">
         <v>302</v>
       </c>
@@ -15910,7 +15883,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="522" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="522" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A522">
         <v>303</v>
       </c>
@@ -15933,7 +15906,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="523" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="523" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A523">
         <v>304</v>
       </c>
@@ -15956,7 +15929,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="524" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="524" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A524">
         <v>305</v>
       </c>
@@ -15979,7 +15952,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="525" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="525" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A525">
         <v>306</v>
       </c>
@@ -16002,7 +15975,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="526" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="526" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A526">
         <v>307</v>
       </c>
@@ -16025,7 +15998,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="527" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="527" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A527">
         <v>308</v>
       </c>
@@ -16048,7 +16021,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="528" spans="1:7" ht="29.15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="528" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A528">
         <v>380</v>
       </c>

</xml_diff>